<commit_message>
journal de bord + math update
</commit_message>
<xml_diff>
--- a/Maths/Moteur_RTX_exercices_2.2.xlsx
+++ b/Maths/Moteur_RTX_exercices_2.2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\univ\but3\math\projet\moteur_RTS\Maths\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20710E11-B4E9-48D8-AF36-08DFC58AFA49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FE75DAB-9327-4192-8043-B8BE4910EE8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="10">
   <si>
     <t>n</t>
   </si>
@@ -50,16 +50,22 @@
     <t>P0</t>
   </si>
   <si>
-    <t>Pdiscret(proie)</t>
+    <t>P-théorique(predateur)</t>
   </si>
   <si>
-    <t>Pdiscret(predateur)</t>
+    <t>P-théorique(proie)</t>
   </si>
   <si>
-    <t>Pthéorique(proie)</t>
+    <t>P-implicite(proie)</t>
   </si>
   <si>
-    <t>Pthéorique(predateur)</t>
+    <t>P-implicite(pred)</t>
+  </si>
+  <si>
+    <t>P-explicite(proie)</t>
+  </si>
+  <si>
+    <t>P-explicite(predateur)</t>
   </si>
 </sst>
 </file>
@@ -129,6 +135,31 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="fr-FR"/>
+              <a:t>Proie</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -169,11 +200,11 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Feuil1!$J$12</c:f>
+              <c:f>Feuil1!$M$12</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Pdiscret(proie)</c:v>
+                  <c:v>P-explicite(proie)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -192,7 +223,7 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Feuil1!$J$13:$J$38</c:f>
+              <c:f>Feuil1!$M$13:$M$38</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="26"/>
@@ -280,7 +311,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-367E-46CD-BC4B-EFE09F2D1488}"/>
+              <c16:uniqueId val="{00000000-651A-4266-ADED-6D4A78B2D759}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -289,11 +320,11 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Feuil1!$K$12</c:f>
+              <c:f>Feuil1!$N$12</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Pdiscret(predateur)</c:v>
+                  <c:v>P-implicite(proie)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -312,7 +343,7 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Feuil1!$K$13:$K$38</c:f>
+              <c:f>Feuil1!$N$13:$N$38</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="26"/>
@@ -320,79 +351,79 @@
                   <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>90</c:v>
+                  <c:v>105.26315789473684</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>81</c:v>
+                  <c:v>110.80332409972297</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>72.900000000000006</c:v>
+                  <c:v>116.63507799970839</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>65.610000000000014</c:v>
+                  <c:v>122.77376631548252</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>59.049000000000021</c:v>
+                  <c:v>129.23554348998158</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>53.144100000000016</c:v>
+                  <c:v>136.03741419998062</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>47.829690000000014</c:v>
+                  <c:v>143.19727810524273</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>43.046721000000012</c:v>
+                  <c:v>150.73397695288708</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>38.742048900000015</c:v>
+                  <c:v>158.66734416093377</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>34.867844010000013</c:v>
+                  <c:v>167.01825701150921</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>31.381059609000019</c:v>
+                  <c:v>175.80869159106228</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>28.242953648100016</c:v>
+                  <c:v>185.06178062217086</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>25.418658283290018</c:v>
+                  <c:v>194.80187433912721</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>22.876792454961013</c:v>
+                  <c:v>205.05460456750231</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>20.589113209464912</c:v>
+                  <c:v>215.84695217631818</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>18.530201888518423</c:v>
+                  <c:v>227.20731808033494</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>16.677181699666583</c:v>
+                  <c:v>239.16559797929992</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>15.009463529699923</c:v>
+                  <c:v>251.753261030842</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>13.508517176729933</c:v>
+                  <c:v>265.00343266404423</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>12.15766545905694</c:v>
+                  <c:v>278.95098175162548</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>10.941898913151247</c:v>
+                  <c:v>293.63261237013205</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>9.8477090218361241</c:v>
+                  <c:v>309.08696038961267</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>8.8629381196525117</c:v>
+                  <c:v>325.35469514696069</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>7.97664430768726</c:v>
+                  <c:v>342.47862647048493</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>7.1789798769185342</c:v>
+                  <c:v>360.50381733735247</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -400,7 +431,127 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-367E-46CD-BC4B-EFE09F2D1488}"/>
+              <c16:uniqueId val="{00000001-651A-4266-ADED-6D4A78B2D759}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Feuil1!$O$12</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>P-théorique(proie)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Feuil1!$O$13:$O$38</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="26"/>
+                <c:pt idx="0">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>105.12710963760242</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>110.51709180756477</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>116.18342427282833</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>122.14027581601701</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>128.40254166877418</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>134.98588075760034</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>141.90675485932579</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>149.18246976412709</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>156.83121854901697</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>164.87212707001291</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>173.32530178673963</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>182.21188003905101</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>191.55408290138976</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>201.37527074704781</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>211.70000166126766</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>222.55409284924696</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>233.96468519259935</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>245.96031111569522</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>258.57096593158491</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>271.82818284590485</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>285.76511180631672</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>300.41660239464363</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>315.81929096897716</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>332.01169227365523</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>349.03429574618463</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-651A-4266-ADED-6D4A78B2D759}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -413,11 +564,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:smooth val="0"/>
-        <c:axId val="225130015"/>
-        <c:axId val="53725231"/>
+        <c:axId val="1653537440"/>
+        <c:axId val="1354027760"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="225130015"/>
+        <c:axId val="1653537440"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -459,7 +610,7 @@
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="53725231"/>
+        <c:crossAx val="1354027760"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -467,7 +618,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="53725231"/>
+        <c:axId val="1354027760"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -518,7 +669,643 @@
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="225130015"/>
+        <c:crossAx val="1653537440"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="fr-FR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="fr-FR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="fr-FR"/>
+              <a:t>prédateur</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Feuil1!$Q$12</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>P-explicite(predateur)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Feuil1!$Q$13:$Q$38</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="26"/>
+                <c:pt idx="0">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>81</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>72.900000000000006</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>65.610000000000014</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>59.049000000000021</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>53.144100000000016</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>47.829690000000014</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>43.046721000000012</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>38.742048900000015</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>34.867844010000013</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>31.381059609000019</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>28.242953648100016</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>25.418658283290018</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>22.876792454961013</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>20.589113209464912</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>18.530201888518423</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>16.677181699666583</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>15.009463529699923</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>13.508517176729933</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>12.15766545905694</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>10.941898913151247</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>9.8477090218361241</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>8.8629381196525117</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>7.97664430768726</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>7.1789798769185342</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-E500-4E04-A9A4-15CB927A01E5}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Feuil1!$R$12</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>P-théorique(predateur)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Feuil1!$R$13:$R$38</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="26"/>
+                <c:pt idx="0">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>90.483741803595947</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>81.873075307798175</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>74.081822068171761</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>67.032004603563905</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>60.653065971263317</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>54.88116360940262</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>49.658530379140927</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>44.932896411722133</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>40.656965974059887</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>36.787944117144207</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>33.287108369807925</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>30.119421191220187</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>27.253179303401236</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>24.659696394160623</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>22.313016014842958</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>20.189651799465519</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18.268352405273443</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>16.529888822158632</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>14.956861922263483</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>13.533528323661251</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>12.245642825298173</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>11.080315836233371</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>10.025884372280357</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>9.0717953289412367</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>8.208499862389866</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-E500-4E04-A9A4-15CB927A01E5}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Feuil1!$S$12</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>P-implicite(pred)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Feuil1!$S$13:$S$38</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="26"/>
+                <c:pt idx="0">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>90.909090909090907</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>82.644628099173545</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>75.131480090157766</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>68.301345536507057</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>62.092132305915506</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>56.44739300537772</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>51.315811823070653</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>46.650738020973321</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>42.409761837248475</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>38.554328942953155</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>35.049389948139229</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>31.863081771035663</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>28.966437973668778</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>26.333125430607979</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>23.939204936916344</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>21.76291357901486</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>19.784466890013508</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>17.985878990921371</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>16.35079908265579</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>14.864362802414352</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>13.513057093103958</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>12.284597357367231</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>11.167815779424755</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>10.15255979947705</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>9.2295998177064096</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-E500-4E04-A9A4-15CB927A01E5}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="1571138064"/>
+        <c:axId val="1354133360"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1571138064"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1354133360"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1354133360"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1571138064"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -645,6 +1432,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
   <cs:axisTitle>
@@ -1161,27 +1988,543 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>454025</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>88900</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>373674</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>3419</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>149225</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>69850</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>61059</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>148004</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Graphique 1">
+        <xdr:cNvPr id="8" name="Graphique 7">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{578CE118-0379-CEA3-9C35-90693B1989A1}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E0A70B44-345A-74F5-2137-6AA93E332A83}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1194,6 +2537,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>350630</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>119270</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>63500</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>129209</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="9" name="Graphique 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BF52C350-3EA6-DFD7-33F0-59F6479D869F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1465,869 +2844,1189 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:N38"/>
+  <dimension ref="B2:S38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>0</v>
       </c>
       <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J2" t="s">
+      <c r="L2" t="s">
         <v>3</v>
       </c>
-      <c r="K2" t="s">
+      <c r="M2" t="s">
         <v>1</v>
       </c>
-      <c r="L2" t="s">
+      <c r="N2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B3">
         <v>0</v>
       </c>
       <c r="C3">
-        <f>$J$3*(($K$3*$L$3+1)^B3)</f>
+        <f>$L$3*(($M$3*$N$3+1)^B3)</f>
         <v>100</v>
       </c>
       <c r="D3">
-        <f>$J$3*(($K$4*$L$3+1)^B3)</f>
+        <f>$L$3*(1/(1-$M$3*$N$3))^B3</f>
         <v>100</v>
       </c>
-      <c r="F3">
-        <f>$J$3*(EXP($K$3*$L$3))^B3</f>
+      <c r="E3">
+        <f>$L$3*(EXP($M$3*$N$3))^B3</f>
         <v>100</v>
       </c>
       <c r="G3">
-        <f>$J$3*(EXP($K$4*$L$3))^B3</f>
+        <f>$L$3*(($M$4*$N$3+1)^B3)</f>
         <v>100</v>
       </c>
-      <c r="J3">
+      <c r="H3">
+        <f>$L$3*(1/(1-$M$4*$N$3))^B3</f>
         <v>100</v>
       </c>
-      <c r="K3">
+      <c r="I3">
+        <f>$L$3*(EXP($M$4*$N$3))^B3</f>
+        <v>100</v>
+      </c>
+      <c r="L3">
+        <v>100</v>
+      </c>
+      <c r="M3">
         <v>0.05</v>
       </c>
-      <c r="L3">
+      <c r="N3">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4">
-        <f t="shared" ref="C4:C8" si="0">$J$3*(($K$3*$L$3+1)^B4)</f>
+        <f>$L$3*(($M$3*$N$3+1)^B4)</f>
         <v>125</v>
       </c>
       <c r="D4">
-        <f t="shared" ref="D4:D8" si="1">$J$3*(($K$4*$L$3+1)^B4)</f>
+        <f>$L$3*(1/(1-$M$3*$N$3))^B4</f>
+        <v>133.33333333333331</v>
+      </c>
+      <c r="E4">
+        <f>$L$3*(EXP($M$3*$N$3))^B4</f>
+        <v>128.40254166877415</v>
+      </c>
+      <c r="G4">
+        <f>$L$3*(($M$4*$N$3+1)^B4)</f>
         <v>50</v>
       </c>
-      <c r="F4">
-        <f t="shared" ref="F4:F7" si="2">$J$3*(EXP($K$3*$L$3))^B4</f>
-        <v>128.40254166877415</v>
-      </c>
-      <c r="G4">
-        <f t="shared" ref="G4:G7" si="3">$J$3*(EXP($K$4*$L$3))^B4</f>
+      <c r="H4">
+        <f>$L$3*(1/(1-$M$4*$N$3))^B4</f>
+        <v>66.666666666666657</v>
+      </c>
+      <c r="I4">
+        <f>$L$3*(EXP($M$4*$N$3))^B4</f>
         <v>60.653065971263345</v>
       </c>
-      <c r="K4">
+      <c r="M4">
         <f>-0.1</f>
         <v>-0.1</v>
       </c>
-      <c r="L4">
+      <c r="N4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B5">
         <v>2</v>
       </c>
       <c r="C5">
-        <f t="shared" si="0"/>
+        <f>$L$3*(($M$3*$N$3+1)^B5)</f>
         <v>156.25</v>
       </c>
       <c r="D5">
-        <f t="shared" si="1"/>
+        <f>$L$3*(1/(1-$M$3*$N$3))^B5</f>
+        <v>177.77777777777777</v>
+      </c>
+      <c r="E5">
+        <f>$L$3*(EXP($M$3*$N$3))^B5</f>
+        <v>164.87212707001279</v>
+      </c>
+      <c r="G5">
+        <f>$L$3*(($M$4*$N$3+1)^B5)</f>
         <v>25</v>
       </c>
-      <c r="F5">
-        <f t="shared" si="2"/>
-        <v>164.87212707001279</v>
-      </c>
-      <c r="G5">
-        <f t="shared" si="3"/>
+      <c r="H5">
+        <f>$L$3*(1/(1-$M$4*$N$3))^B5</f>
+        <v>44.444444444444443</v>
+      </c>
+      <c r="I5">
+        <f>$L$3*(EXP($M$4*$N$3))^B5</f>
         <v>36.787944117144235</v>
       </c>
-      <c r="L5">
+      <c r="N5">
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B6">
         <v>3</v>
       </c>
       <c r="C6">
-        <f t="shared" si="0"/>
+        <f>$L$3*(($M$3*$N$3+1)^B6)</f>
         <v>195.3125</v>
       </c>
       <c r="D6">
-        <f t="shared" si="1"/>
+        <f>$L$3*(1/(1-$M$3*$N$3))^B6</f>
+        <v>237.03703703703701</v>
+      </c>
+      <c r="E6">
+        <f>$L$3*(EXP($M$3*$N$3))^B6</f>
+        <v>211.70000166126744</v>
+      </c>
+      <c r="G6">
+        <f>$L$3*(($M$4*$N$3+1)^B6)</f>
         <v>12.5</v>
       </c>
-      <c r="F6">
-        <f t="shared" si="2"/>
-        <v>211.70000166126744</v>
-      </c>
-      <c r="G6">
-        <f t="shared" si="3"/>
+      <c r="H6">
+        <f>$L$3*(1/(1-$M$4*$N$3))^B6</f>
+        <v>29.629629629629626</v>
+      </c>
+      <c r="I6">
+        <f>$L$3*(EXP($M$4*$N$3))^B6</f>
         <v>22.313016014842983</v>
       </c>
-      <c r="L6">
+      <c r="N6">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B7">
         <v>4</v>
       </c>
       <c r="C7">
-        <f t="shared" si="0"/>
+        <f>$L$3*(($M$3*$N$3+1)^B7)</f>
         <v>244.140625</v>
       </c>
       <c r="D7">
-        <f t="shared" si="1"/>
+        <f>$L$3*(1/(1-$M$3*$N$3))^B7</f>
+        <v>316.04938271604937</v>
+      </c>
+      <c r="E7">
+        <f>$L$3*(EXP($M$3*$N$3))^B7</f>
+        <v>271.82818284590445</v>
+      </c>
+      <c r="G7">
+        <f>$L$3*(($M$4*$N$3+1)^B7)</f>
         <v>6.25</v>
       </c>
-      <c r="F7">
-        <f t="shared" si="2"/>
-        <v>271.82818284590445</v>
-      </c>
-      <c r="G7">
-        <f t="shared" si="3"/>
+      <c r="H7">
+        <f>$L$3*(1/(1-$M$4*$N$3))^B7</f>
+        <v>19.753086419753085</v>
+      </c>
+      <c r="I7">
+        <f>$L$3*(EXP($M$4*$N$3))^B7</f>
         <v>13.533528323661271</v>
       </c>
     </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B8">
         <v>5</v>
       </c>
       <c r="C8">
-        <f t="shared" si="0"/>
+        <f>$L$3*(($M$3*$N$3+1)^B8)</f>
         <v>305.17578125</v>
       </c>
       <c r="D8">
-        <f t="shared" si="1"/>
+        <f>$L$3*(1/(1-$M$3*$N$3))^B8</f>
+        <v>421.39917695473247</v>
+      </c>
+      <c r="E8">
+        <f>$L$3*(EXP($M$3*$N$3))^B8</f>
+        <v>349.03429574618406</v>
+      </c>
+      <c r="G8">
+        <f>$L$3*(($M$4*$N$3+1)^B8)</f>
         <v>3.125</v>
       </c>
-      <c r="F8">
-        <f>$J$3*(EXP($K$3*$L$3))^B8</f>
-        <v>349.03429574618406</v>
-      </c>
-      <c r="G8">
-        <f>$J$3*(EXP($K$4*$L$3))^B8</f>
+      <c r="H8">
+        <f>$L$3*(1/(1-$M$4*$N$3))^B8</f>
+        <v>13.16872427983539</v>
+      </c>
+      <c r="I8">
+        <f>$L$3*(EXP($M$4*$N$3))^B8</f>
         <v>8.2084998623898802</v>
       </c>
     </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>0</v>
       </c>
       <c r="C12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" t="s">
+        <v>6</v>
+      </c>
+      <c r="E12" t="s">
+        <v>5</v>
+      </c>
+      <c r="G12" t="s">
+        <v>9</v>
+      </c>
+      <c r="H12" t="s">
+        <v>7</v>
+      </c>
+      <c r="I12" t="s">
         <v>4</v>
       </c>
-      <c r="D12" t="s">
+      <c r="L12" t="s">
+        <v>0</v>
+      </c>
+      <c r="M12" t="s">
+        <v>8</v>
+      </c>
+      <c r="N12" t="s">
+        <v>6</v>
+      </c>
+      <c r="O12" t="s">
         <v>5</v>
       </c>
-      <c r="F12" t="s">
-        <v>6</v>
-      </c>
-      <c r="G12" t="s">
+      <c r="Q12" t="s">
+        <v>9</v>
+      </c>
+      <c r="R12" t="s">
+        <v>4</v>
+      </c>
+      <c r="S12" t="s">
         <v>7</v>
       </c>
-      <c r="I12" t="s">
-        <v>0</v>
-      </c>
-      <c r="J12" t="s">
-        <v>4</v>
-      </c>
-      <c r="K12" t="s">
-        <v>5</v>
-      </c>
-      <c r="M12" t="s">
-        <v>6</v>
-      </c>
-      <c r="N12" t="s">
-        <v>7</v>
-      </c>
     </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B13">
         <v>0</v>
       </c>
       <c r="C13">
-        <f>$J$3*(($K$3*$L$5+1)^B13)</f>
+        <f>$L$3*(($M$3*$N$5+1)^B13)</f>
         <v>100</v>
       </c>
       <c r="D13">
-        <f>$J$3*(($K$4*$L$5+1)^B13)</f>
+        <f>$L$3*(1/(1-$M$3*$N$5))^B13</f>
         <v>100</v>
       </c>
-      <c r="F13">
-        <f>$J$3*(EXP($K$3*$L$5))^B13</f>
+      <c r="E13">
+        <f>$L$3*(EXP($M$3*$N$5))^B13</f>
         <v>100</v>
       </c>
       <c r="G13">
-        <f>$J$3*(EXP($K$4*$L$5))^B13</f>
+        <f>$L$3*(($M$4*$N$5+1)^B13)</f>
         <v>100</v>
       </c>
+      <c r="H13">
+        <f>$L$3*(1/(1-$M$4*$N$5))^B13</f>
+        <v>100</v>
+      </c>
       <c r="I13">
+        <f>$L$3*(EXP($M$4*$N$5))^B13</f>
+        <v>100</v>
+      </c>
+      <c r="L13">
         <v>0</v>
       </c>
-      <c r="J13">
-        <f>$J$3*(($K$3*$L$4+1)^I13)</f>
+      <c r="M13">
+        <f>$L$3*(($M$3*$N$4+1)^L13)</f>
         <v>100</v>
       </c>
-      <c r="K13">
-        <f>$J$3*(($K$4*$L$4+1)^I13)</f>
+      <c r="N13">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L13</f>
         <v>100</v>
       </c>
-      <c r="M13">
-        <f>$J$3*(EXP($K$3*$L$4))^I13</f>
+      <c r="O13">
+        <f>$L$3*(EXP($M$3*$N$4))^L13</f>
         <v>100</v>
       </c>
-      <c r="N13">
-        <f>$J$3*(EXP($K$4*$L$4))^I13</f>
+      <c r="Q13">
+        <f>$L$3*(($M$4*$N$4+1)^L13)</f>
         <v>100</v>
       </c>
+      <c r="R13">
+        <f>$L$3*(EXP($M$4*$N$4))^L13</f>
+        <v>100</v>
+      </c>
+      <c r="S13">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L13</f>
+        <v>100</v>
+      </c>
     </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B14">
         <v>1</v>
       </c>
       <c r="C14">
-        <f>$J$3*(($K$3*$L$5+1)^B14)</f>
+        <f>$L$3*(($M$3*$N$5+1)^B14)</f>
         <v>225</v>
       </c>
       <c r="D14">
-        <f>$J$3*(($K$4*$L$5+1)^B14)</f>
+        <f>$L$3*(1/(1-$M$3*$N$5))^B14</f>
+        <v>-400</v>
+      </c>
+      <c r="E14">
+        <f>$L$3*(EXP($M$3*$N$5))^B14</f>
+        <v>349.03429574618417</v>
+      </c>
+      <c r="G14">
+        <f>$L$3*(($M$4*$N$5+1)^B14)</f>
         <v>-150</v>
       </c>
-      <c r="F14">
-        <f>$J$3*(EXP($K$3*$L$5))^B14</f>
-        <v>349.03429574618417</v>
-      </c>
-      <c r="G14">
-        <f>$J$3*(EXP($K$4*$L$5))^B14</f>
+      <c r="H14">
+        <f>$L$3*(1/(1-$M$4*$N$5))^B14</f>
+        <v>28.571428571428569</v>
+      </c>
+      <c r="I14">
+        <f>$L$3*(EXP($M$4*$N$5))^B14</f>
         <v>8.2084998623898802</v>
       </c>
-      <c r="I14">
+      <c r="L14">
         <v>1</v>
       </c>
-      <c r="J14">
-        <f t="shared" ref="J14:J38" si="4">$J$3*(($K$3*$L$4+1)^I14)</f>
+      <c r="M14">
+        <f>$L$3*(($M$3*$N$4+1)^L14)</f>
         <v>105</v>
       </c>
-      <c r="K14">
-        <f t="shared" ref="K14:K38" si="5">$J$3*(($K$4*$L$4+1)^I14)</f>
+      <c r="N14">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L14</f>
+        <v>105.26315789473684</v>
+      </c>
+      <c r="O14">
+        <f>$L$3*(EXP($M$3*$N$4))^L14</f>
+        <v>105.12710963760242</v>
+      </c>
+      <c r="Q14">
+        <f>$L$3*(($M$4*$N$4+1)^L14)</f>
         <v>90</v>
       </c>
-      <c r="M14">
-        <f t="shared" ref="M14:M38" si="6">$J$3*(EXP($K$3*$L$4))^I14</f>
-        <v>105.12710963760242</v>
-      </c>
-      <c r="N14">
-        <f t="shared" ref="N14:N38" si="7">$J$3*(EXP($K$4*$L$4))^I14</f>
+      <c r="R14">
+        <f>$L$3*(EXP($M$4*$N$4))^L14</f>
         <v>90.483741803595947</v>
       </c>
+      <c r="S14">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L14</f>
+        <v>90.909090909090907</v>
+      </c>
     </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="I15">
+    <row r="15" spans="2:19" x14ac:dyDescent="0.35">
+      <c r="L15">
         <v>2</v>
       </c>
-      <c r="J15">
-        <f t="shared" si="4"/>
+      <c r="M15">
+        <f>$L$3*(($M$3*$N$4+1)^L15)</f>
         <v>110.25</v>
       </c>
-      <c r="K15">
-        <f t="shared" si="5"/>
+      <c r="N15">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L15</f>
+        <v>110.80332409972297</v>
+      </c>
+      <c r="O15">
+        <f>$L$3*(EXP($M$3*$N$4))^L15</f>
+        <v>110.51709180756477</v>
+      </c>
+      <c r="Q15">
+        <f>$L$3*(($M$4*$N$4+1)^L15)</f>
         <v>81</v>
       </c>
-      <c r="M15">
-        <f t="shared" si="6"/>
-        <v>110.51709180756477</v>
-      </c>
-      <c r="N15">
-        <f t="shared" si="7"/>
+      <c r="R15">
+        <f>$L$3*(EXP($M$4*$N$4))^L15</f>
         <v>81.873075307798175</v>
       </c>
+      <c r="S15">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L15</f>
+        <v>82.644628099173545</v>
+      </c>
     </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="I16">
+    <row r="16" spans="2:19" x14ac:dyDescent="0.35">
+      <c r="L16">
         <v>3</v>
       </c>
-      <c r="J16">
-        <f t="shared" si="4"/>
+      <c r="M16">
+        <f>$L$3*(($M$3*$N$4+1)^L16)</f>
         <v>115.76250000000002</v>
       </c>
-      <c r="K16">
-        <f t="shared" si="5"/>
+      <c r="N16">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L16</f>
+        <v>116.63507799970839</v>
+      </c>
+      <c r="O16">
+        <f>$L$3*(EXP($M$3*$N$4))^L16</f>
+        <v>116.18342427282833</v>
+      </c>
+      <c r="Q16">
+        <f>$L$3*(($M$4*$N$4+1)^L16)</f>
         <v>72.900000000000006</v>
       </c>
-      <c r="M16">
-        <f t="shared" si="6"/>
-        <v>116.18342427282833</v>
-      </c>
-      <c r="N16">
-        <f t="shared" si="7"/>
+      <c r="R16">
+        <f>$L$3*(EXP($M$4*$N$4))^L16</f>
         <v>74.081822068171761</v>
       </c>
+      <c r="S16">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L16</f>
+        <v>75.131480090157766</v>
+      </c>
     </row>
-    <row r="17" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
         <v>0</v>
       </c>
       <c r="C17" t="s">
+        <v>8</v>
+      </c>
+      <c r="D17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E17" t="s">
+        <v>5</v>
+      </c>
+      <c r="G17" t="s">
+        <v>9</v>
+      </c>
+      <c r="H17" t="s">
+        <v>7</v>
+      </c>
+      <c r="I17" t="s">
         <v>4</v>
       </c>
-      <c r="D17" t="s">
-        <v>5</v>
-      </c>
-      <c r="F17" t="s">
-        <v>6</v>
-      </c>
-      <c r="G17" t="s">
-        <v>7</v>
-      </c>
-      <c r="I17">
+      <c r="L17">
         <v>4</v>
       </c>
-      <c r="J17">
-        <f t="shared" si="4"/>
+      <c r="M17">
+        <f>$L$3*(($M$3*$N$4+1)^L17)</f>
         <v>121.550625</v>
       </c>
-      <c r="K17">
-        <f t="shared" si="5"/>
+      <c r="N17">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L17</f>
+        <v>122.77376631548252</v>
+      </c>
+      <c r="O17">
+        <f>$L$3*(EXP($M$3*$N$4))^L17</f>
+        <v>122.14027581601701</v>
+      </c>
+      <c r="Q17">
+        <f>$L$3*(($M$4*$N$4+1)^L17)</f>
         <v>65.610000000000014</v>
       </c>
-      <c r="M17">
-        <f t="shared" si="6"/>
-        <v>122.14027581601701</v>
-      </c>
-      <c r="N17">
-        <f t="shared" si="7"/>
+      <c r="R17">
+        <f>$L$3*(EXP($M$4*$N$4))^L17</f>
         <v>67.032004603563905</v>
       </c>
+      <c r="S17">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L17</f>
+        <v>68.301345536507057</v>
+      </c>
     </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B18">
         <v>0</v>
       </c>
       <c r="C18">
-        <f>$J$3*(($K$3*$L$6+1)^B18)</f>
+        <f>$L$3*(($M$3*$N$6+1)^B18)</f>
         <v>100</v>
       </c>
       <c r="D18">
-        <f>$J$3*(($K$4*$L$6+1)^B18)</f>
+        <f>$L$3*(1/(1-$M$3*$N$6))^B18</f>
         <v>100</v>
       </c>
-      <c r="F18">
-        <f>$J$3*(EXP($K$3*$L$6))^B18</f>
+      <c r="E18">
+        <f>$L$3*(EXP($M$3*$N$6))^B18</f>
         <v>100</v>
       </c>
       <c r="G18">
-        <f>$J$3*(EXP($K$4*$L$6))^B18</f>
+        <f>$L$3*(($M$4*$N$6+1)^B18)</f>
         <v>100</v>
       </c>
+      <c r="H18">
+        <f>$L$3*(1/(1-$M$4*$N$6))^B18</f>
+        <v>100</v>
+      </c>
       <c r="I18">
+        <f>$L$3*(EXP($M$4*$N$6))^B18</f>
+        <v>100</v>
+      </c>
+      <c r="L18">
         <v>5</v>
       </c>
-      <c r="J18">
-        <f t="shared" si="4"/>
+      <c r="M18">
+        <f>$L$3*(($M$3*$N$4+1)^L18)</f>
         <v>127.62815625000002</v>
       </c>
-      <c r="K18">
-        <f t="shared" si="5"/>
+      <c r="N18">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L18</f>
+        <v>129.23554348998158</v>
+      </c>
+      <c r="O18">
+        <f>$L$3*(EXP($M$3*$N$4))^L18</f>
+        <v>128.40254166877418</v>
+      </c>
+      <c r="Q18">
+        <f>$L$3*(($M$4*$N$4+1)^L18)</f>
         <v>59.049000000000021</v>
       </c>
-      <c r="M18">
-        <f t="shared" si="6"/>
-        <v>128.40254166877418</v>
-      </c>
-      <c r="N18">
-        <f t="shared" si="7"/>
+      <c r="R18">
+        <f>$L$3*(EXP($M$4*$N$4))^L18</f>
         <v>60.653065971263317</v>
       </c>
+      <c r="S18">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L18</f>
+        <v>62.092132305915506</v>
+      </c>
     </row>
-    <row r="19" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B19">
         <v>1</v>
       </c>
       <c r="C19">
-        <f t="shared" ref="C19:C20" si="8">$J$3*(($K$3*$L$6+1)^B19)</f>
+        <f>$L$3*(($M$3*$N$6+1)^B19)</f>
         <v>175</v>
       </c>
       <c r="D19">
-        <f t="shared" ref="D19:D20" si="9">$J$3*(($K$4*$L$6+1)^B19)</f>
+        <f>$L$3*(1/(1-$M$3*$N$6))^B19</f>
+        <v>400</v>
+      </c>
+      <c r="E19">
+        <f>$L$3*(EXP($M$3*$N$6))^B19</f>
+        <v>211.70000166126749</v>
+      </c>
+      <c r="G19">
+        <f>$L$3*(($M$4*$N$6+1)^B19)</f>
         <v>-50</v>
       </c>
-      <c r="F19">
-        <f t="shared" ref="F19:F20" si="10">$J$3*(EXP($K$3*$L$6))^B19</f>
-        <v>211.70000166126749</v>
-      </c>
-      <c r="G19">
-        <f t="shared" ref="G19:G20" si="11">$J$3*(EXP($K$4*$L$6))^B19</f>
+      <c r="H19">
+        <f>$L$3*(1/(1-$M$4*$N$6))^B19</f>
+        <v>40</v>
+      </c>
+      <c r="I19">
+        <f>$L$3*(EXP($M$4*$N$6))^B19</f>
         <v>22.313016014842983</v>
       </c>
-      <c r="I19">
+      <c r="L19">
         <v>6</v>
       </c>
-      <c r="J19">
-        <f t="shared" si="4"/>
+      <c r="M19">
+        <f>$L$3*(($M$3*$N$4+1)^L19)</f>
         <v>134.0095640625</v>
       </c>
-      <c r="K19">
-        <f t="shared" si="5"/>
+      <c r="N19">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L19</f>
+        <v>136.03741419998062</v>
+      </c>
+      <c r="O19">
+        <f>$L$3*(EXP($M$3*$N$4))^L19</f>
+        <v>134.98588075760034</v>
+      </c>
+      <c r="Q19">
+        <f>$L$3*(($M$4*$N$4+1)^L19)</f>
         <v>53.144100000000016</v>
       </c>
-      <c r="M19">
-        <f t="shared" si="6"/>
-        <v>134.98588075760034</v>
-      </c>
-      <c r="N19">
-        <f t="shared" si="7"/>
+      <c r="R19">
+        <f>$L$3*(EXP($M$4*$N$4))^L19</f>
         <v>54.88116360940262</v>
       </c>
+      <c r="S19">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L19</f>
+        <v>56.44739300537772</v>
+      </c>
     </row>
-    <row r="20" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B20">
         <v>2</v>
       </c>
       <c r="C20">
-        <f t="shared" si="8"/>
+        <f>$L$3*(($M$3*$N$6+1)^B20)</f>
         <v>306.25</v>
       </c>
       <c r="D20">
-        <f t="shared" si="9"/>
+        <f>$L$3*(1/(1-$M$3*$N$6))^B20</f>
+        <v>1600</v>
+      </c>
+      <c r="E20">
+        <f>$L$3*(EXP($M$3*$N$6))^B20</f>
+        <v>448.16890703380653</v>
+      </c>
+      <c r="G20">
+        <f>$L$3*(($M$4*$N$6+1)^B20)</f>
         <v>25</v>
       </c>
-      <c r="F20">
-        <f t="shared" si="10"/>
-        <v>448.16890703380653</v>
-      </c>
-      <c r="G20">
-        <f t="shared" si="11"/>
+      <c r="H20">
+        <f>$L$3*(1/(1-$M$4*$N$6))^B20</f>
+        <v>16.000000000000004</v>
+      </c>
+      <c r="I20">
+        <f>$L$3*(EXP($M$4*$N$6))^B20</f>
         <v>4.9787068367863938</v>
       </c>
-      <c r="I20">
+      <c r="L20">
         <v>7</v>
       </c>
-      <c r="J20">
-        <f t="shared" si="4"/>
+      <c r="M20">
+        <f>$L$3*(($M$3*$N$4+1)^L20)</f>
         <v>140.71004226562502</v>
       </c>
-      <c r="K20">
-        <f t="shared" si="5"/>
+      <c r="N20">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L20</f>
+        <v>143.19727810524273</v>
+      </c>
+      <c r="O20">
+        <f>$L$3*(EXP($M$3*$N$4))^L20</f>
+        <v>141.90675485932579</v>
+      </c>
+      <c r="Q20">
+        <f>$L$3*(($M$4*$N$4+1)^L20)</f>
         <v>47.829690000000014</v>
       </c>
-      <c r="M20">
-        <f t="shared" si="6"/>
-        <v>141.90675485932579</v>
-      </c>
-      <c r="N20">
-        <f t="shared" si="7"/>
+      <c r="R20">
+        <f>$L$3*(EXP($M$4*$N$4))^L20</f>
         <v>49.658530379140927</v>
       </c>
+      <c r="S20">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L20</f>
+        <v>51.315811823070653</v>
+      </c>
     </row>
-    <row r="21" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="I21">
+    <row r="21" spans="2:19" x14ac:dyDescent="0.35">
+      <c r="L21">
         <v>8</v>
       </c>
-      <c r="J21">
-        <f t="shared" si="4"/>
+      <c r="M21">
+        <f>$L$3*(($M$3*$N$4+1)^L21)</f>
         <v>147.74554437890626</v>
       </c>
-      <c r="K21">
-        <f t="shared" si="5"/>
+      <c r="N21">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L21</f>
+        <v>150.73397695288708</v>
+      </c>
+      <c r="O21">
+        <f>$L$3*(EXP($M$3*$N$4))^L21</f>
+        <v>149.18246976412709</v>
+      </c>
+      <c r="Q21">
+        <f>$L$3*(($M$4*$N$4+1)^L21)</f>
         <v>43.046721000000012</v>
       </c>
-      <c r="M21">
-        <f t="shared" si="6"/>
-        <v>149.18246976412709</v>
-      </c>
-      <c r="N21">
-        <f t="shared" si="7"/>
+      <c r="R21">
+        <f>$L$3*(EXP($M$4*$N$4))^L21</f>
         <v>44.932896411722133</v>
       </c>
+      <c r="S21">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L21</f>
+        <v>46.650738020973321</v>
+      </c>
     </row>
-    <row r="22" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="I22">
+    <row r="22" spans="2:19" x14ac:dyDescent="0.35">
+      <c r="L22">
         <v>9</v>
       </c>
-      <c r="J22">
-        <f t="shared" si="4"/>
+      <c r="M22">
+        <f>$L$3*(($M$3*$N$4+1)^L22)</f>
         <v>155.13282159785157</v>
       </c>
-      <c r="K22">
-        <f t="shared" si="5"/>
+      <c r="N22">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L22</f>
+        <v>158.66734416093377</v>
+      </c>
+      <c r="O22">
+        <f>$L$3*(EXP($M$3*$N$4))^L22</f>
+        <v>156.83121854901697</v>
+      </c>
+      <c r="Q22">
+        <f>$L$3*(($M$4*$N$4+1)^L22)</f>
         <v>38.742048900000015</v>
       </c>
-      <c r="M22">
-        <f t="shared" si="6"/>
-        <v>156.83121854901697</v>
-      </c>
-      <c r="N22">
-        <f t="shared" si="7"/>
+      <c r="R22">
+        <f>$L$3*(EXP($M$4*$N$4))^L22</f>
         <v>40.656965974059887</v>
       </c>
+      <c r="S22">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L22</f>
+        <v>42.409761837248475</v>
+      </c>
     </row>
-    <row r="23" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="I23">
+    <row r="23" spans="2:19" x14ac:dyDescent="0.35">
+      <c r="L23">
         <v>10</v>
       </c>
-      <c r="J23">
-        <f t="shared" si="4"/>
+      <c r="M23">
+        <f>$L$3*(($M$3*$N$4+1)^L23)</f>
         <v>162.88946267774415</v>
       </c>
-      <c r="K23">
-        <f t="shared" si="5"/>
+      <c r="N23">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L23</f>
+        <v>167.01825701150921</v>
+      </c>
+      <c r="O23">
+        <f>$L$3*(EXP($M$3*$N$4))^L23</f>
+        <v>164.87212707001291</v>
+      </c>
+      <c r="Q23">
+        <f>$L$3*(($M$4*$N$4+1)^L23)</f>
         <v>34.867844010000013</v>
       </c>
-      <c r="M23">
-        <f t="shared" si="6"/>
-        <v>164.87212707001291</v>
-      </c>
-      <c r="N23">
-        <f t="shared" si="7"/>
+      <c r="R23">
+        <f>$L$3*(EXP($M$4*$N$4))^L23</f>
         <v>36.787944117144207</v>
       </c>
+      <c r="S23">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L23</f>
+        <v>38.554328942953155</v>
+      </c>
     </row>
-    <row r="24" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="I24">
+    <row r="24" spans="2:19" x14ac:dyDescent="0.35">
+      <c r="L24">
         <v>11</v>
       </c>
-      <c r="J24">
-        <f t="shared" si="4"/>
+      <c r="M24">
+        <f>$L$3*(($M$3*$N$4+1)^L24)</f>
         <v>171.03393581163138</v>
       </c>
-      <c r="K24">
-        <f t="shared" si="5"/>
+      <c r="N24">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L24</f>
+        <v>175.80869159106228</v>
+      </c>
+      <c r="O24">
+        <f>$L$3*(EXP($M$3*$N$4))^L24</f>
+        <v>173.32530178673963</v>
+      </c>
+      <c r="Q24">
+        <f>$L$3*(($M$4*$N$4+1)^L24)</f>
         <v>31.381059609000019</v>
       </c>
-      <c r="M24">
-        <f t="shared" si="6"/>
-        <v>173.32530178673963</v>
-      </c>
-      <c r="N24">
-        <f t="shared" si="7"/>
+      <c r="R24">
+        <f>$L$3*(EXP($M$4*$N$4))^L24</f>
         <v>33.287108369807925</v>
       </c>
+      <c r="S24">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L24</f>
+        <v>35.049389948139229</v>
+      </c>
     </row>
-    <row r="25" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="I25">
+    <row r="25" spans="2:19" x14ac:dyDescent="0.35">
+      <c r="L25">
         <v>12</v>
       </c>
-      <c r="J25">
-        <f t="shared" si="4"/>
+      <c r="M25">
+        <f>$L$3*(($M$3*$N$4+1)^L25)</f>
         <v>179.58563260221291</v>
       </c>
-      <c r="K25">
-        <f t="shared" si="5"/>
+      <c r="N25">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L25</f>
+        <v>185.06178062217086</v>
+      </c>
+      <c r="O25">
+        <f>$L$3*(EXP($M$3*$N$4))^L25</f>
+        <v>182.21188003905101</v>
+      </c>
+      <c r="Q25">
+        <f>$L$3*(($M$4*$N$4+1)^L25)</f>
         <v>28.242953648100016</v>
       </c>
-      <c r="M25">
-        <f t="shared" si="6"/>
-        <v>182.21188003905101</v>
-      </c>
-      <c r="N25">
-        <f t="shared" si="7"/>
+      <c r="R25">
+        <f>$L$3*(EXP($M$4*$N$4))^L25</f>
         <v>30.119421191220187</v>
       </c>
+      <c r="S25">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L25</f>
+        <v>31.863081771035663</v>
+      </c>
     </row>
-    <row r="26" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="I26">
+    <row r="26" spans="2:19" x14ac:dyDescent="0.35">
+      <c r="L26">
         <v>13</v>
       </c>
-      <c r="J26">
-        <f t="shared" si="4"/>
+      <c r="M26">
+        <f>$L$3*(($M$3*$N$4+1)^L26)</f>
         <v>188.56491423232359</v>
       </c>
-      <c r="K26">
-        <f t="shared" si="5"/>
+      <c r="N26">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L26</f>
+        <v>194.80187433912721</v>
+      </c>
+      <c r="O26">
+        <f>$L$3*(EXP($M$3*$N$4))^L26</f>
+        <v>191.55408290138976</v>
+      </c>
+      <c r="Q26">
+        <f>$L$3*(($M$4*$N$4+1)^L26)</f>
         <v>25.418658283290018</v>
       </c>
-      <c r="M26">
-        <f t="shared" si="6"/>
-        <v>191.55408290138976</v>
-      </c>
-      <c r="N26">
-        <f t="shared" si="7"/>
+      <c r="R26">
+        <f>$L$3*(EXP($M$4*$N$4))^L26</f>
         <v>27.253179303401236</v>
       </c>
+      <c r="S26">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L26</f>
+        <v>28.966437973668778</v>
+      </c>
     </row>
-    <row r="27" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="I27">
+    <row r="27" spans="2:19" x14ac:dyDescent="0.35">
+      <c r="L27">
         <v>14</v>
       </c>
-      <c r="J27">
-        <f t="shared" si="4"/>
+      <c r="M27">
+        <f>$L$3*(($M$3*$N$4+1)^L27)</f>
         <v>197.99315994393973</v>
       </c>
-      <c r="K27">
-        <f t="shared" si="5"/>
+      <c r="N27">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L27</f>
+        <v>205.05460456750231</v>
+      </c>
+      <c r="O27">
+        <f>$L$3*(EXP($M$3*$N$4))^L27</f>
+        <v>201.37527074704781</v>
+      </c>
+      <c r="Q27">
+        <f>$L$3*(($M$4*$N$4+1)^L27)</f>
         <v>22.876792454961013</v>
       </c>
-      <c r="M27">
-        <f t="shared" si="6"/>
-        <v>201.37527074704781</v>
-      </c>
-      <c r="N27">
-        <f t="shared" si="7"/>
+      <c r="R27">
+        <f>$L$3*(EXP($M$4*$N$4))^L27</f>
         <v>24.659696394160623</v>
       </c>
+      <c r="S27">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L27</f>
+        <v>26.333125430607979</v>
+      </c>
     </row>
-    <row r="28" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="I28">
+    <row r="28" spans="2:19" x14ac:dyDescent="0.35">
+      <c r="L28">
         <v>15</v>
       </c>
-      <c r="J28">
-        <f t="shared" si="4"/>
+      <c r="M28">
+        <f>$L$3*(($M$3*$N$4+1)^L28)</f>
         <v>207.8928179411368</v>
       </c>
-      <c r="K28">
-        <f t="shared" si="5"/>
+      <c r="N28">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L28</f>
+        <v>215.84695217631818</v>
+      </c>
+      <c r="O28">
+        <f>$L$3*(EXP($M$3*$N$4))^L28</f>
+        <v>211.70000166126766</v>
+      </c>
+      <c r="Q28">
+        <f>$L$3*(($M$4*$N$4+1)^L28)</f>
         <v>20.589113209464912</v>
       </c>
-      <c r="M28">
-        <f t="shared" si="6"/>
-        <v>211.70000166126766</v>
-      </c>
-      <c r="N28">
-        <f t="shared" si="7"/>
+      <c r="R28">
+        <f>$L$3*(EXP($M$4*$N$4))^L28</f>
         <v>22.313016014842958</v>
       </c>
+      <c r="S28">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L28</f>
+        <v>23.939204936916344</v>
+      </c>
     </row>
-    <row r="29" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="I29">
+    <row r="29" spans="2:19" x14ac:dyDescent="0.35">
+      <c r="L29">
         <v>16</v>
       </c>
-      <c r="J29">
-        <f t="shared" si="4"/>
+      <c r="M29">
+        <f>$L$3*(($M$3*$N$4+1)^L29)</f>
         <v>218.2874588381936</v>
       </c>
-      <c r="K29">
-        <f t="shared" si="5"/>
+      <c r="N29">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L29</f>
+        <v>227.20731808033494</v>
+      </c>
+      <c r="O29">
+        <f>$L$3*(EXP($M$3*$N$4))^L29</f>
+        <v>222.55409284924696</v>
+      </c>
+      <c r="Q29">
+        <f>$L$3*(($M$4*$N$4+1)^L29)</f>
         <v>18.530201888518423</v>
       </c>
-      <c r="M29">
-        <f t="shared" si="6"/>
-        <v>222.55409284924696</v>
-      </c>
-      <c r="N29">
-        <f t="shared" si="7"/>
+      <c r="R29">
+        <f>$L$3*(EXP($M$4*$N$4))^L29</f>
         <v>20.189651799465519</v>
       </c>
+      <c r="S29">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L29</f>
+        <v>21.76291357901486</v>
+      </c>
     </row>
-    <row r="30" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="I30">
+    <row r="30" spans="2:19" x14ac:dyDescent="0.35">
+      <c r="L30">
         <v>17</v>
       </c>
-      <c r="J30">
-        <f t="shared" si="4"/>
+      <c r="M30">
+        <f>$L$3*(($M$3*$N$4+1)^L30)</f>
         <v>229.2018317801033</v>
       </c>
-      <c r="K30">
-        <f t="shared" si="5"/>
+      <c r="N30">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L30</f>
+        <v>239.16559797929992</v>
+      </c>
+      <c r="O30">
+        <f>$L$3*(EXP($M$3*$N$4))^L30</f>
+        <v>233.96468519259935</v>
+      </c>
+      <c r="Q30">
+        <f>$L$3*(($M$4*$N$4+1)^L30)</f>
         <v>16.677181699666583</v>
       </c>
-      <c r="M30">
-        <f t="shared" si="6"/>
-        <v>233.96468519259935</v>
-      </c>
-      <c r="N30">
-        <f t="shared" si="7"/>
+      <c r="R30">
+        <f>$L$3*(EXP($M$4*$N$4))^L30</f>
         <v>18.268352405273443</v>
       </c>
+      <c r="S30">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L30</f>
+        <v>19.784466890013508</v>
+      </c>
     </row>
-    <row r="31" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="I31">
+    <row r="31" spans="2:19" x14ac:dyDescent="0.35">
+      <c r="L31">
         <v>18</v>
       </c>
-      <c r="J31">
-        <f t="shared" si="4"/>
+      <c r="M31">
+        <f>$L$3*(($M$3*$N$4+1)^L31)</f>
         <v>240.66192336910848</v>
       </c>
-      <c r="K31">
-        <f t="shared" si="5"/>
+      <c r="N31">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L31</f>
+        <v>251.753261030842</v>
+      </c>
+      <c r="O31">
+        <f>$L$3*(EXP($M$3*$N$4))^L31</f>
+        <v>245.96031111569522</v>
+      </c>
+      <c r="Q31">
+        <f>$L$3*(($M$4*$N$4+1)^L31)</f>
         <v>15.009463529699923</v>
       </c>
-      <c r="M31">
-        <f t="shared" si="6"/>
-        <v>245.96031111569522</v>
-      </c>
-      <c r="N31">
-        <f t="shared" si="7"/>
+      <c r="R31">
+        <f>$L$3*(EXP($M$4*$N$4))^L31</f>
         <v>16.529888822158632</v>
       </c>
+      <c r="S31">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L31</f>
+        <v>17.985878990921371</v>
+      </c>
     </row>
-    <row r="32" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="I32">
+    <row r="32" spans="2:19" x14ac:dyDescent="0.35">
+      <c r="L32">
         <v>19</v>
       </c>
-      <c r="J32">
-        <f t="shared" si="4"/>
+      <c r="M32">
+        <f>$L$3*(($M$3*$N$4+1)^L32)</f>
         <v>252.69501953756389</v>
       </c>
-      <c r="K32">
-        <f t="shared" si="5"/>
+      <c r="N32">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L32</f>
+        <v>265.00343266404423</v>
+      </c>
+      <c r="O32">
+        <f>$L$3*(EXP($M$3*$N$4))^L32</f>
+        <v>258.57096593158491</v>
+      </c>
+      <c r="Q32">
+        <f>$L$3*(($M$4*$N$4+1)^L32)</f>
         <v>13.508517176729933</v>
       </c>
-      <c r="M32">
-        <f t="shared" si="6"/>
-        <v>258.57096593158491</v>
-      </c>
-      <c r="N32">
-        <f t="shared" si="7"/>
+      <c r="R32">
+        <f>$L$3*(EXP($M$4*$N$4))^L32</f>
         <v>14.956861922263483</v>
       </c>
+      <c r="S32">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L32</f>
+        <v>16.35079908265579</v>
+      </c>
     </row>
-    <row r="33" spans="9:14" x14ac:dyDescent="0.35">
-      <c r="I33">
+    <row r="33" spans="12:19" x14ac:dyDescent="0.35">
+      <c r="L33">
         <v>20</v>
       </c>
-      <c r="J33">
-        <f t="shared" si="4"/>
+      <c r="M33">
+        <f>$L$3*(($M$3*$N$4+1)^L33)</f>
         <v>265.32977051444209</v>
       </c>
-      <c r="K33">
-        <f t="shared" si="5"/>
+      <c r="N33">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L33</f>
+        <v>278.95098175162548</v>
+      </c>
+      <c r="O33">
+        <f>$L$3*(EXP($M$3*$N$4))^L33</f>
+        <v>271.82818284590485</v>
+      </c>
+      <c r="Q33">
+        <f>$L$3*(($M$4*$N$4+1)^L33)</f>
         <v>12.15766545905694</v>
       </c>
-      <c r="M33">
-        <f t="shared" si="6"/>
-        <v>271.82818284590485</v>
-      </c>
-      <c r="N33">
-        <f t="shared" si="7"/>
+      <c r="R33">
+        <f>$L$3*(EXP($M$4*$N$4))^L33</f>
         <v>13.533528323661251</v>
       </c>
+      <c r="S33">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L33</f>
+        <v>14.864362802414352</v>
+      </c>
     </row>
-    <row r="34" spans="9:14" x14ac:dyDescent="0.35">
-      <c r="I34">
+    <row r="34" spans="12:19" x14ac:dyDescent="0.35">
+      <c r="L34">
         <v>21</v>
       </c>
-      <c r="J34">
-        <f>$J$3*(($K$3*$L$4+1)^I34)</f>
+      <c r="M34">
+        <f>$L$3*(($M$3*$N$4+1)^L34)</f>
         <v>278.59625904016417</v>
       </c>
-      <c r="K34">
-        <f>$J$3*(($K$4*$L$4+1)^I34)</f>
+      <c r="N34">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L34</f>
+        <v>293.63261237013205</v>
+      </c>
+      <c r="O34">
+        <f>$L$3*(EXP($M$3*$N$4))^L34</f>
+        <v>285.76511180631672</v>
+      </c>
+      <c r="Q34">
+        <f>$L$3*(($M$4*$N$4+1)^L34)</f>
         <v>10.941898913151247</v>
       </c>
-      <c r="M34">
-        <f>$J$3*(EXP($K$3*$L$4))^I34</f>
-        <v>285.76511180631672</v>
-      </c>
-      <c r="N34">
-        <f>$J$3*(EXP($K$4*$L$4))^I34</f>
+      <c r="R34">
+        <f>$L$3*(EXP($M$4*$N$4))^L34</f>
         <v>12.245642825298173</v>
       </c>
+      <c r="S34">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L34</f>
+        <v>13.513057093103958</v>
+      </c>
     </row>
-    <row r="35" spans="9:14" x14ac:dyDescent="0.35">
-      <c r="I35">
+    <row r="35" spans="12:19" x14ac:dyDescent="0.35">
+      <c r="L35">
         <v>22</v>
       </c>
-      <c r="J35">
-        <f t="shared" si="4"/>
+      <c r="M35">
+        <f>$L$3*(($M$3*$N$4+1)^L35)</f>
         <v>292.52607199217238</v>
       </c>
-      <c r="K35">
-        <f t="shared" si="5"/>
+      <c r="N35">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L35</f>
+        <v>309.08696038961267</v>
+      </c>
+      <c r="O35">
+        <f>$L$3*(EXP($M$3*$N$4))^L35</f>
+        <v>300.41660239464363</v>
+      </c>
+      <c r="Q35">
+        <f>$L$3*(($M$4*$N$4+1)^L35)</f>
         <v>9.8477090218361241</v>
       </c>
-      <c r="M35">
-        <f t="shared" si="6"/>
-        <v>300.41660239464363</v>
-      </c>
-      <c r="N35">
-        <f t="shared" si="7"/>
+      <c r="R35">
+        <f>$L$3*(EXP($M$4*$N$4))^L35</f>
         <v>11.080315836233371</v>
       </c>
+      <c r="S35">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L35</f>
+        <v>12.284597357367231</v>
+      </c>
     </row>
-    <row r="36" spans="9:14" x14ac:dyDescent="0.35">
-      <c r="I36">
+    <row r="36" spans="12:19" x14ac:dyDescent="0.35">
+      <c r="L36">
         <v>23</v>
       </c>
-      <c r="J36">
-        <f t="shared" si="4"/>
+      <c r="M36">
+        <f>$L$3*(($M$3*$N$4+1)^L36)</f>
         <v>307.15237559178104</v>
       </c>
-      <c r="K36">
-        <f t="shared" si="5"/>
+      <c r="N36">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L36</f>
+        <v>325.35469514696069</v>
+      </c>
+      <c r="O36">
+        <f>$L$3*(EXP($M$3*$N$4))^L36</f>
+        <v>315.81929096897716</v>
+      </c>
+      <c r="Q36">
+        <f>$L$3*(($M$4*$N$4+1)^L36)</f>
         <v>8.8629381196525117</v>
       </c>
-      <c r="M36">
-        <f t="shared" si="6"/>
-        <v>315.81929096897716</v>
-      </c>
-      <c r="N36">
-        <f t="shared" si="7"/>
+      <c r="R36">
+        <f>$L$3*(EXP($M$4*$N$4))^L36</f>
         <v>10.025884372280357</v>
       </c>
+      <c r="S36">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L36</f>
+        <v>11.167815779424755</v>
+      </c>
     </row>
-    <row r="37" spans="9:14" x14ac:dyDescent="0.35">
-      <c r="I37">
+    <row r="37" spans="12:19" x14ac:dyDescent="0.35">
+      <c r="L37">
         <v>24</v>
       </c>
-      <c r="J37">
-        <f t="shared" si="4"/>
+      <c r="M37">
+        <f>$L$3*(($M$3*$N$4+1)^L37)</f>
         <v>322.50999437137006</v>
       </c>
-      <c r="K37">
-        <f t="shared" si="5"/>
+      <c r="N37">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L37</f>
+        <v>342.47862647048493</v>
+      </c>
+      <c r="O37">
+        <f>$L$3*(EXP($M$3*$N$4))^L37</f>
+        <v>332.01169227365523</v>
+      </c>
+      <c r="Q37">
+        <f>$L$3*(($M$4*$N$4+1)^L37)</f>
         <v>7.97664430768726</v>
       </c>
-      <c r="M37">
-        <f t="shared" si="6"/>
-        <v>332.01169227365523</v>
-      </c>
-      <c r="N37">
-        <f t="shared" si="7"/>
+      <c r="R37">
+        <f>$L$3*(EXP($M$4*$N$4))^L37</f>
         <v>9.0717953289412367</v>
       </c>
+      <c r="S37">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L37</f>
+        <v>10.15255979947705</v>
+      </c>
     </row>
-    <row r="38" spans="9:14" x14ac:dyDescent="0.35">
-      <c r="I38">
+    <row r="38" spans="12:19" x14ac:dyDescent="0.35">
+      <c r="L38">
         <v>25</v>
       </c>
-      <c r="J38">
-        <f t="shared" si="4"/>
+      <c r="M38">
+        <f>$L$3*(($M$3*$N$4+1)^L38)</f>
         <v>338.63549408993856</v>
       </c>
-      <c r="K38">
-        <f t="shared" si="5"/>
+      <c r="N38">
+        <f>$L$3*(1/(1-$M$3*$N$4))^L38</f>
+        <v>360.50381733735247</v>
+      </c>
+      <c r="O38">
+        <f>$L$3*(EXP($M$3*$N$4))^L38</f>
+        <v>349.03429574618463</v>
+      </c>
+      <c r="Q38">
+        <f>$L$3*(($M$4*$N$4+1)^L38)</f>
         <v>7.1789798769185342</v>
       </c>
-      <c r="M38">
-        <f t="shared" si="6"/>
-        <v>349.03429574618463</v>
-      </c>
-      <c r="N38">
-        <f t="shared" si="7"/>
+      <c r="R38">
+        <f>$L$3*(EXP($M$4*$N$4))^L38</f>
         <v>8.208499862389866</v>
+      </c>
+      <c r="S38">
+        <f>$L$3*(1/(1-$M$4*$N$4))^L38</f>
+        <v>9.2295998177064096</v>
       </c>
     </row>
   </sheetData>

</xml_diff>